<commit_message>
writing updates, other may motif updates
</commit_message>
<xml_diff>
--- a/MEME manual annotations.xlsx
+++ b/MEME manual annotations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enoch/Documents/Local Erill Research/drippy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC81E372-4697-0448-82CF-383D040B701F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37520687-95FE-4F48-8E2A-841F655509B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15640" yWindow="760" windowWidth="13760" windowHeight="18360" xr2:uid="{7AA2DFE4-5D5E-2F4D-BE0F-FA5793F0E76F}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{7AA2DFE4-5D5E-2F4D-BE0F-FA5793F0E76F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -285,7 +285,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -299,8 +299,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,6 +317,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -344,10 +357,10 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -685,6 +698,7 @@
   <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="20.1640625" customWidth="1"/>
     <col min="6" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
@@ -695,7 +709,7 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D1" t="s">
@@ -707,16 +721,16 @@
       <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1202,22 +1216,21 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
+      <c r="A19">
         <v>2</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19">
         <v>8</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" t="s">
         <v>31</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" t="s">
         <v>32</v>
       </c>
-      <c r="F19" s="2"/>
       <c r="G19" t="s">
         <v>75</v>
       </c>
@@ -1238,7 +1251,7 @@
       <c r="B20">
         <v>9</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" t="s">
         <v>5</v>
       </c>
       <c r="G20" t="s">
@@ -1261,7 +1274,7 @@
       <c r="B21">
         <v>10</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" t="s">
         <v>5</v>
       </c>
       <c r="G21" t="s">
@@ -1284,7 +1297,7 @@
       <c r="B22">
         <v>1</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" t="s">
         <v>5</v>
       </c>
       <c r="G22" t="s">
@@ -1307,7 +1320,7 @@
       <c r="B23">
         <v>2</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" t="s">
         <v>5</v>
       </c>
       <c r="F23" t="s">
@@ -1333,7 +1346,7 @@
       <c r="B24">
         <v>3</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" t="s">
         <v>5</v>
       </c>
       <c r="G24" t="s">
@@ -1356,7 +1369,7 @@
       <c r="B25">
         <v>4</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" t="s">
         <v>6</v>
       </c>
       <c r="D25" t="s">
@@ -1388,7 +1401,7 @@
       <c r="B26">
         <v>5</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" t="s">
         <v>5</v>
       </c>
       <c r="G26" t="s">
@@ -1411,7 +1424,7 @@
       <c r="B27">
         <v>6</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" t="s">
         <v>6</v>
       </c>
       <c r="D27" t="s">
@@ -1443,7 +1456,7 @@
       <c r="B28">
         <v>7</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" t="s">
         <v>6</v>
       </c>
       <c r="D28" t="s">
@@ -1472,7 +1485,7 @@
       <c r="B29">
         <v>8</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" t="s">
         <v>5</v>
       </c>
       <c r="G29" t="s">
@@ -1495,7 +1508,7 @@
       <c r="B30">
         <v>9</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" t="s">
         <v>5</v>
       </c>
       <c r="G30" t="s">
@@ -1518,7 +1531,7 @@
       <c r="B31">
         <v>10</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" t="s">
         <v>5</v>
       </c>
       <c r="F31" t="s">
@@ -1544,7 +1557,7 @@
       <c r="B32">
         <v>1</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" t="s">
         <v>5</v>
       </c>
       <c r="F32" t="s">
@@ -1570,7 +1583,7 @@
       <c r="B33">
         <v>2</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" t="s">
         <v>5</v>
       </c>
       <c r="G33" t="s">
@@ -1593,7 +1606,7 @@
       <c r="B34">
         <v>3</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" t="s">
         <v>5</v>
       </c>
       <c r="G34" t="s">
@@ -1616,7 +1629,7 @@
       <c r="B35">
         <v>4</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" t="s">
         <v>5</v>
       </c>
       <c r="F35" t="s">
@@ -1642,7 +1655,7 @@
       <c r="B36">
         <v>5</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" t="s">
         <v>6</v>
       </c>
       <c r="D36" t="s">
@@ -1671,7 +1684,7 @@
       <c r="B37">
         <v>6</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" t="s">
         <v>6</v>
       </c>
       <c r="D37" t="s">
@@ -1703,7 +1716,7 @@
       <c r="B38">
         <v>7</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" t="s">
         <v>5</v>
       </c>
       <c r="F38" t="s">
@@ -1729,7 +1742,7 @@
       <c r="B39">
         <v>8</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" t="s">
         <v>5</v>
       </c>
       <c r="G39" t="s">
@@ -1752,7 +1765,7 @@
       <c r="B40">
         <v>9</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" t="s">
         <v>5</v>
       </c>
       <c r="G40" t="s">
@@ -1775,7 +1788,7 @@
       <c r="B41">
         <v>10</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" t="s">
         <v>5</v>
       </c>
       <c r="G41" t="s">

</xml_diff>